<commit_message>
Add find minimum in rotated sorted array solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4573,6 +4573,51 @@
       <c r="I91" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/find-rotation-count.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Find Minimum in Rotated Sorted Array</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/find-minimum-rotated-sorted-array.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add single non-duplicate element in sorted array solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I92"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4618,6 +4618,51 @@
       <c r="I92" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/find-minimum-rotated-sorted-array.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Single Non-Duplicate Element in a Sorted Array</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/single-non-duplicate.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add find peak element solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I93"/>
+  <dimension ref="A1:I94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4663,6 +4663,51 @@
       <c r="I93" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/single-non-duplicate.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Find Peak Element</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/find-peak-element.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add integer square root solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:I95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4708,6 +4708,51 @@
       <c r="I94" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/find-peak-element.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Integer Square Root (Floor, Binary Search)</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/sqrt-integer.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add N-th root solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I95"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4753,6 +4753,51 @@
       <c r="I95" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/sqrt-integer.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>N-th Root of a Number (Integer, Binary Search)</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/nth-root.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Koko eating bananas solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4798,6 +4798,51 @@
       <c r="I96" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/nth-root.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Koko Eating Bananas (Minimum Eating Speed)</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/koko-eating-bananas.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add minimum days to make m bouquets solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4843,6 +4843,51 @@
       <c r="I97" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/koko-eating-bananas.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Minimum Number of Days to Make M Bouquets</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/minimum-days-to-make-bouquets.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add smallest divisor given a threshold solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I98"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4888,6 +4888,51 @@
       <c r="I98" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/minimum-days-to-make-bouquets.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Smallest Divisor Given a Threshold</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/smallest-divisor-threshold.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add kth missing positive number solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I99"/>
+  <dimension ref="A1:I100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4933,6 +4933,51 @@
       <c r="I99" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/smallest-divisor-threshold.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Kth Missing Positive Number (Brute Force)</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/kth-missing-positive-number.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add kth missing positive number (binary search) solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4978,6 +4978,51 @@
       <c r="I100" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/kth-missing-positive-number.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Kth Missing Positive Number (Binary Search, O(log n))</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/kth-missing-positive-number-binary-search.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log ship-within-days in tracker and questions log
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5023,6 +5023,51 @@
       <c r="I101" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/kth-missing-positive-number-binary-search.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Capacity To Ship Packages Within D Days</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/ship-within-days.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add aggressive cows solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I102"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5068,6 +5068,51 @@
       <c r="I102" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/ship-within-days.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Aggressive Cows (Maximize Minimum Distance)</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/aggressive-cows.py</t>
         </is>
       </c>
     </row>
@@ -5133,22 +5178,22 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>pattern-printing</t>
+          <t>binary-search</t>
         </is>
       </c>
       <c r="B7" s="2">
-        <f>COUNTIF(Questions!B:B,"pattern-printing")</f>
+        <f>COUNTIF(Questions!B:B,"binary-search")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>binary-search</t>
+          <t>pattern-printing</t>
         </is>
       </c>
       <c r="B8" s="2">
-        <f>COUNTIF(Questions!B:B,"binary-search")</f>
+        <f>COUNTIF(Questions!B:B,"pattern-printing")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add allocate minimum pages solution and note
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5113,6 +5113,51 @@
       <c r="I103" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/aggressive-cows.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Allocate Minimum Pages (Book Allocation)</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/allocate-minimum-pages.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark 15 solutions with failing edge cases as struggled for review
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
@@ -3937,7 +3937,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F79" s="2" t="n">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F89" s="2" t="n">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>struggled</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add split array largest sum solution and note
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I104"/>
+  <dimension ref="A1:I105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5158,6 +5158,51 @@
       <c r="I104" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/allocate-minimum-pages.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Split Array Largest Sum</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/split-array-largest-sum.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add painter's partition solution and note
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5203,6 +5203,51 @@
       <c r="I105" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/split-array-largest-sum.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Painter's Partition (Minimum Time)</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/painters-partition.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add gas station min-max distance solution and notes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5248,6 +5248,51 @@
       <c r="I106" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/painters-partition.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Minimise Maximum Distance Between Gas Stations (Real-Valued Binary Search)</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/gas-station-min-max-distance.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add median of two sorted arrays solution, flagged struggled, with notes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I107"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5293,6 +5293,51 @@
       <c r="I107" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/gas-station-min-max-distance.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Median of Two Sorted Arrays (Merge Walk)</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>struggled</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/median-of-two-sorted-arrays.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update median of two sorted arrays with the tie fix, mark solved
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -5319,11 +5319,11 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>struggled</t>
+          <t>solved</t>
         </is>
       </c>
       <c r="F108" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add row with maximum number of 1s solution
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5338,6 +5338,51 @@
       <c r="I108" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/median-of-two-sorted-arrays.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Row with Maximum Number of 1s</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>matrix</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>solutions/matrix/row-with-max-ones.py</t>
         </is>
       </c>
     </row>
@@ -5458,22 +5503,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>sliding-window</t>
+          <t>matrix</t>
         </is>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF(Questions!B:B,"sliding-window")</f>
+        <f>COUNTIF(Questions!B:B,"matrix")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>matrix</t>
+          <t>sliding-window</t>
         </is>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(Questions!B:B,"matrix")</f>
+        <f>COUNTIF(Questions!B:B,"sliding-window")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add sorted-row binary search variant of row-with-max-ones
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5383,6 +5383,51 @@
       <c r="I109" s="2" t="inlineStr">
         <is>
           <t>solutions/matrix/row-with-max-ones.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Row with Maximum 1s (Sorted Rows, Binary Search per Row)</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>matrix</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>solutions/matrix/row-with-max-ones-sorted-binary-search.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add search 2D matrix solution and note
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I110"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5428,6 +5428,51 @@
       <c r="I110" s="2" t="inlineStr">
         <is>
           <t>solutions/matrix/row-with-max-ones-sorted-binary-search.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Search a 2D Matrix (Rows Sorted, Next Row Starts After Previous Ends)</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>matrix</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>solutions/matrix/search-2d-matrix.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add search 2D matrix II solution and note
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I111"/>
+  <dimension ref="A1:I112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5473,6 +5473,51 @@
       <c r="I111" s="2" t="inlineStr">
         <is>
           <t>solutions/matrix/search-2d-matrix.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Search a 2D Matrix II (Rows and Columns Sorted, Top-Right Walk)</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>matrix</t>
+        </is>
+      </c>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>solutions/matrix/search-2d-matrix-ii.py</t>
         </is>
       </c>
     </row>
@@ -5571,33 +5616,33 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>matrix</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <f>COUNTIF(Questions!B:B,"matrix")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>recursion</t>
         </is>
       </c>
-      <c r="B10" s="2">
+      <c r="B11" s="2">
         <f>COUNTIF(Questions!B:B,"recursion")</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>two-pointers</t>
-        </is>
-      </c>
-      <c r="B11" s="2">
-        <f>COUNTIF(Questions!B:B,"two-pointers")</f>
-        <v/>
-      </c>
-    </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>matrix</t>
+          <t>two-pointers</t>
         </is>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF(Questions!B:B,"matrix")</f>
+        <f>COUNTIF(Questions!B:B,"two-pointers")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add find peak element II solution and notes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I112"/>
+  <dimension ref="A1:I113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5518,6 +5518,51 @@
       <c r="I112" s="2" t="inlineStr">
         <is>
           <t>solutions/matrix/search-2d-matrix-ii.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Find Peak Element II (Binary Search on Columns)</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/find-peak-element-ii.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add matrix median solution (with high=mid-1 fix) and notes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I113"/>
+  <dimension ref="A1:I114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5563,6 +5563,51 @@
       <c r="I113" s="2" t="inlineStr">
         <is>
           <t>solutions/binary-search/find-peak-element-ii.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Median of a Row-Wise Sorted Matrix (Binary Search on Value)</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>binary-search</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>solutions/binary-search/matrix-median.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add remove outermost parentheses solution and strings notes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I114"/>
+  <dimension ref="A1:I115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5611,6 +5611,51 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Remove Outermost Parentheses</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>strings</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>solutions/strings/remove-outer-parentheses.py</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5622,7 +5667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5758,6 +5803,17 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>strings</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(Questions!B:B,"strings")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add maximum nesting depth of parentheses solution and notes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5653,6 +5653,51 @@
       <c r="I115" s="2" t="inlineStr">
         <is>
           <t>solutions/strings/remove-outer-parentheses.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Maximum Nesting Depth of the Parentheses</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>strings</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>solutions/strings/max-nesting-depth-parentheses.py</t>
         </is>
       </c>
     </row>
@@ -5795,22 +5840,22 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>intervals</t>
+          <t>strings</t>
         </is>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(Questions!B:B,"intervals")</f>
+        <f>COUNTIF(Questions!B:B,"strings")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>strings</t>
+          <t>intervals</t>
         </is>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF(Questions!B:B,"strings")</f>
+        <f>COUNTIF(Questions!B:B,"intervals")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add roman to integer solution and notes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I116"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5698,6 +5698,51 @@
       <c r="I116" s="2" t="inlineStr">
         <is>
           <t>solutions/strings/max-nesting-depth-parentheses.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Roman to Integer</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>strings</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>solutions/strings/roman-to-integer.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add string to integer (atoi) solution and notes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I117"/>
+  <dimension ref="A1:I118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5743,6 +5743,51 @@
       <c r="I117" s="2" t="inlineStr">
         <is>
           <t>solutions/strings/roman-to-integer.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>String to Integer (atoi)</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>strings</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>solutions/strings/string-to-integer-atoi.py</t>
         </is>
       </c>
     </row>
@@ -5874,22 +5919,22 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>sliding-window</t>
+          <t>strings</t>
         </is>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(Questions!B:B,"sliding-window")</f>
+        <f>COUNTIF(Questions!B:B,"strings")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>strings</t>
+          <t>sliding-window</t>
         </is>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(Questions!B:B,"strings")</f>
+        <f>COUNTIF(Questions!B:B,"sliding-window")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add longest palindromic substring solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I118"/>
+  <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5788,6 +5788,51 @@
       <c r="I118" s="2" t="inlineStr">
         <is>
           <t>solutions/strings/string-to-integer-atoi.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Longest Palindromic Substring (Expand Around Center)</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>strings</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>solutions/strings/longest-palindromic-substring.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add sum of beauty of all substrings solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I119"/>
+  <dimension ref="A1:I120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5833,6 +5833,51 @@
       <c r="I119" s="2" t="inlineStr">
         <is>
           <t>solutions/strings/longest-palindromic-substring.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Sum of Beauty of All Substrings</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>strings</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>solutions/strings/sum-of-beauty-of-all-substrings.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add count complete substrings solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I120"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5878,6 +5878,51 @@
       <c r="I120" s="2" t="inlineStr">
         <is>
           <t>solutions/strings/sum-of-beauty-of-all-substrings.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Count Complete Substrings (Fixed-Length Sliding Windows)</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>strings</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>solutions/strings/count-complete-substrings.py</t>
         </is>
       </c>
     </row>
@@ -5987,33 +6032,33 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>strings</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <f>COUNTIF(Questions!B:B,"strings")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>recursion</t>
         </is>
       </c>
-      <c r="B11" s="2">
+      <c r="B12" s="2">
         <f>COUNTIF(Questions!B:B,"recursion")</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>two-pointers</t>
-        </is>
-      </c>
-      <c r="B12" s="2">
-        <f>COUNTIF(Questions!B:B,"two-pointers")</f>
-        <v/>
-      </c>
-    </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>strings</t>
+          <t>two-pointers</t>
         </is>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(Questions!B:B,"strings")</f>
+        <f>COUNTIF(Questions!B:B,"two-pointers")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add LeetCode set matrix zeroes solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:I122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5884,43 +5884,88 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
+          <t>Set Matrix Zeroes (LeetCode, In Place)</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>matrix</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>solutions/matrix/set-matrix-zeroes-leetcode.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Count Complete Substrings (Fixed-Length Sliding Windows)</t>
         </is>
       </c>
-      <c r="B121" s="2" t="inlineStr">
+      <c r="B122" s="2" t="inlineStr">
         <is>
           <t>strings</t>
         </is>
       </c>
-      <c r="C121" s="5" t="inlineStr">
+      <c r="C122" s="5" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="D121" s="2" t="inlineStr">
+      <c r="D122" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>solved</t>
-        </is>
-      </c>
-      <c r="F121" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G121" s="2" t="inlineStr">
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H121" s="2" t="inlineStr">
+      <c r="H122" s="2" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="I121" s="2" t="inlineStr">
+      <c r="I122" s="2" t="inlineStr">
         <is>
           <t>solutions/strings/count-complete-substrings.py</t>
         </is>

</xml_diff>

<commit_message>
Add pow(x, n) solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I122"/>
+  <dimension ref="A1:I123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5929,43 +5929,88 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
+          <t>Pow(x, n) (Binary Exponentiation)</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/pow-x-n.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
           <t>Count Complete Substrings (Fixed-Length Sliding Windows)</t>
         </is>
       </c>
-      <c r="B122" s="2" t="inlineStr">
+      <c r="B123" s="2" t="inlineStr">
         <is>
           <t>strings</t>
         </is>
       </c>
-      <c r="C122" s="5" t="inlineStr">
+      <c r="C123" s="5" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="D122" s="2" t="inlineStr">
+      <c r="D123" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="E122" s="2" t="inlineStr">
-        <is>
-          <t>solved</t>
-        </is>
-      </c>
-      <c r="F122" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G122" s="2" t="inlineStr">
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H122" s="2" t="inlineStr">
+      <c r="H123" s="2" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="I122" s="2" t="inlineStr">
+      <c r="I123" s="2" t="inlineStr">
         <is>
           <t>solutions/strings/count-complete-substrings.py</t>
         </is>
@@ -6077,22 +6122,22 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>strings</t>
+          <t>recursion</t>
         </is>
       </c>
       <c r="B11" s="2">
-        <f>COUNTIF(Questions!B:B,"strings")</f>
+        <f>COUNTIF(Questions!B:B,"recursion")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>recursion</t>
+          <t>strings</t>
         </is>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF(Questions!B:B,"recursion")</f>
+        <f>COUNTIF(Questions!B:B,"strings")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add generate parentheses solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I123"/>
+  <dimension ref="A1:I124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6013,6 +6013,51 @@
       <c r="I123" s="2" t="inlineStr">
         <is>
           <t>solutions/strings/count-complete-substrings.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Generate Parentheses (Backtracking with Open/Close Counts)</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/generate-parentheses.py</t>
         </is>
       </c>
     </row>
@@ -6111,22 +6156,22 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>matrix</t>
+          <t>recursion</t>
         </is>
       </c>
       <c r="B10" s="2">
-        <f>COUNTIF(Questions!B:B,"matrix")</f>
+        <f>COUNTIF(Questions!B:B,"recursion")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>recursion</t>
+          <t>matrix</t>
         </is>
       </c>
       <c r="B11" s="2">
-        <f>COUNTIF(Questions!B:B,"recursion")</f>
+        <f>COUNTIF(Questions!B:B,"matrix")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add power set solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I124"/>
+  <dimension ref="A1:I125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6058,6 +6058,51 @@
       <c r="I124" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/generate-parentheses.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Power Set (Pick / Not-Pick Subsequences)</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/power-set.py</t>
         </is>
       </c>
     </row>
@@ -6145,22 +6190,22 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>math-geometry</t>
+          <t>recursion</t>
         </is>
       </c>
       <c r="B9" s="2">
-        <f>COUNTIF(Questions!B:B,"math-geometry")</f>
+        <f>COUNTIF(Questions!B:B,"recursion")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>recursion</t>
+          <t>math-geometry</t>
         </is>
       </c>
       <c r="B10" s="2">
-        <f>COUNTIF(Questions!B:B,"recursion")</f>
+        <f>COUNTIF(Questions!B:B,"math-geometry")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add count good numbers solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I125"/>
+  <dimension ref="A1:I126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6103,6 +6103,51 @@
       <c r="I125" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/power-set.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Count Good Numbers (Modular Fast Power)</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/count-good-numbers.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add reverse a stack solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I126"/>
+  <dimension ref="A1:I127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6148,6 +6148,51 @@
       <c r="I126" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/count-good-numbers.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Reverse a Stack (Pop Into a Second List)</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/reverse-a-stack.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add subsequence sum K exists solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I127"/>
+  <dimension ref="A1:I128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6193,6 +6193,51 @@
       <c r="I127" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/reverse-a-stack.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Check if a Subsequence With Sum K Exists (Recursion With Pruning)</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/subsequence-sum-k-exists.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add count subsequences with sum K solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I128"/>
+  <dimension ref="A1:I129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6238,6 +6238,51 @@
       <c r="I128" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/subsequence-sum-k-exists.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Count Subsequences With Sum K (Recursion, Returns Counts)</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/count-subsequences-sum-k.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add binary strings with no adjacent zeros solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I129"/>
+  <dimension ref="A1:I130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6283,6 +6283,51 @@
       <c r="I129" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/count-subsequences-sum-k.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Generate Binary Strings With No Adjacent Zeros</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/binary-strings-no-adjacent-zeros.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add combination sum solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I130"/>
+  <dimension ref="A1:I131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6328,6 +6328,51 @@
       <c r="I130" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/binary-strings-no-adjacent-zeros.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Combination Sum (Reuse Allowed, Pick / Not-Pick)</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C131" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/combination-sum.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add combination sum II solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I131"/>
+  <dimension ref="A1:I132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6373,6 +6373,51 @@
       <c r="I131" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/combination-sum.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Combination Sum II (Each Number Once, Skip Equal Groups)</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/combination-sum-ii.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add subsets solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I132"/>
+  <dimension ref="A1:I133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6418,6 +6418,51 @@
       <c r="I132" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/combination-sum-ii.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Subsets I (All Subsets of Distinct Numbers)</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/subsets.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add subsets II solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I133"/>
+  <dimension ref="A1:I134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6463,6 +6463,51 @@
       <c r="I133" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/subsets.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Subsets II (All Subsets With Duplicates)</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/subsets-ii.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add combination sum III solution and notes
</commit_message>
<xml_diff>
--- a/questions-log.xlsx
+++ b/questions-log.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I134"/>
+  <dimension ref="A1:I135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6508,6 +6508,51 @@
       <c r="I134" s="2" t="inlineStr">
         <is>
           <t>solutions/recursion/subsets-ii.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Combination Sum III (Exactly K Numbers From 1-9)</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>recursion</t>
+        </is>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>solved</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>solutions/recursion/combination-sum-iii.py</t>
         </is>
       </c>
     </row>

</xml_diff>